<commit_message>
Actualiza backups y reorganizacion de historicos
</commit_message>
<xml_diff>
--- a/SIGA-Backup/07_docentes.xlsx
+++ b/SIGA-Backup/07_docentes.xlsx
@@ -397,11 +397,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F6"/>
+  <dimension ref="A1:F14"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
-    <col min="2" max="2" width="16.83203125" customWidth="1"/>
-    <col min="3" max="3" width="15.83203125" customWidth="1"/>
+    <col min="2" max="2" width="18.83203125" customWidth="1"/>
+    <col min="3" max="3" width="29.83203125" customWidth="1"/>
     <col min="4" max="4" width="19.83203125" customWidth="1"/>
     <col min="5" max="5" width="12.83203125" customWidth="1"/>
     <col min="6" max="6" width="10.83203125" customWidth="1"/>
@@ -449,33 +449,33 @@
     </row>
     <row r="3">
       <c r="A3">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="B3" t="str">
-        <v>González</v>
+        <v>Gerbán</v>
       </c>
       <c r="C3" t="str">
-        <v>Eugenia Luz</v>
+        <v>Patricia- Fernández Claudia</v>
       </c>
       <c r="D3" t="str">
-        <v>eugeluz@gmail.com</v>
+        <v/>
       </c>
       <c r="E3" t="str">
-        <v>3814744362</v>
-      </c>
-      <c r="F3">
-        <v>23141145</v>
+        <v/>
+      </c>
+      <c r="F3" t="str">
+        <v/>
       </c>
     </row>
     <row r="4">
       <c r="A4">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="B4" t="str">
-        <v>Sin</v>
+        <v>Gerbán</v>
       </c>
       <c r="C4" t="str">
-        <v>Asignar</v>
+        <v>Patricia</v>
       </c>
       <c r="D4" t="str">
         <v/>
@@ -489,47 +489,207 @@
     </row>
     <row r="5">
       <c r="A5">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B5" t="str">
-        <v>Soler</v>
+        <v>González</v>
       </c>
       <c r="C5" t="str">
-        <v>Federico</v>
+        <v>Eugenia Luz</v>
       </c>
       <c r="D5" t="str">
-        <v/>
+        <v>eugeluz@gmail.com</v>
       </c>
       <c r="E5" t="str">
-        <v/>
-      </c>
-      <c r="F5" t="str">
-        <v/>
+        <v>3814744362</v>
+      </c>
+      <c r="F5">
+        <v>23141145</v>
       </c>
     </row>
     <row r="6">
       <c r="A6">
+        <v>9</v>
+      </c>
+      <c r="B6" t="str">
+        <v>Gutierrez</v>
+      </c>
+      <c r="C6" t="str">
+        <v>Silvia Cristina</v>
+      </c>
+      <c r="D6" t="str">
+        <v/>
+      </c>
+      <c r="E6" t="str">
+        <v/>
+      </c>
+      <c r="F6" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7">
+        <v>13</v>
+      </c>
+      <c r="B7" t="str">
+        <v>Ilardo</v>
+      </c>
+      <c r="C7" t="str">
+        <v>Selva</v>
+      </c>
+      <c r="D7" t="str">
+        <v/>
+      </c>
+      <c r="E7" t="str">
+        <v/>
+      </c>
+      <c r="F7" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8">
+        <v>10</v>
+      </c>
+      <c r="B8" t="str">
+        <v>Moyano</v>
+      </c>
+      <c r="C8" t="str">
+        <v>Rossana</v>
+      </c>
+      <c r="D8" t="str">
+        <v/>
+      </c>
+      <c r="E8" t="str">
+        <v/>
+      </c>
+      <c r="F8" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9">
+        <v>8</v>
+      </c>
+      <c r="B9" t="str">
+        <v>Navas</v>
+      </c>
+      <c r="C9" t="str">
+        <v>Hugo Edgar</v>
+      </c>
+      <c r="D9" t="str">
+        <v/>
+      </c>
+      <c r="E9" t="str">
+        <v/>
+      </c>
+      <c r="F9" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10">
+        <v>7</v>
+      </c>
+      <c r="B10" t="str">
+        <v>Ocaranza Zavalia</v>
+      </c>
+      <c r="C10" t="str">
+        <v>Manuel</v>
+      </c>
+      <c r="D10" t="str">
+        <v/>
+      </c>
+      <c r="E10" t="str">
+        <v/>
+      </c>
+      <c r="F10" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11">
+        <v>6</v>
+      </c>
+      <c r="B11" t="str">
+        <v>Orellana</v>
+      </c>
+      <c r="C11" t="str">
+        <v>Marcela Rosa</v>
+      </c>
+      <c r="D11" t="str">
+        <v/>
+      </c>
+      <c r="E11" t="str">
+        <v/>
+      </c>
+      <c r="F11" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12">
+        <v>5</v>
+      </c>
+      <c r="B12" t="str">
+        <v>Sin</v>
+      </c>
+      <c r="C12" t="str">
+        <v>Asignar</v>
+      </c>
+      <c r="D12" t="str">
+        <v/>
+      </c>
+      <c r="E12" t="str">
+        <v/>
+      </c>
+      <c r="F12" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13">
+        <v>2</v>
+      </c>
+      <c r="B13" t="str">
+        <v>Soler</v>
+      </c>
+      <c r="C13" t="str">
+        <v>Federico</v>
+      </c>
+      <c r="D13" t="str">
+        <v/>
+      </c>
+      <c r="E13" t="str">
+        <v/>
+      </c>
+      <c r="F13" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14">
         <v>4</v>
       </c>
-      <c r="B6" t="str">
+      <c r="B14" t="str">
         <v>Susana Ramallo</v>
       </c>
-      <c r="C6" t="str">
+      <c r="C14" t="str">
         <v>Mendez Sergio</v>
       </c>
-      <c r="D6" t="str">
-        <v/>
-      </c>
-      <c r="E6" t="str">
-        <v/>
-      </c>
-      <c r="F6" t="str">
+      <c r="D14" t="str">
+        <v/>
+      </c>
+      <c r="E14" t="str">
+        <v/>
+      </c>
+      <c r="F14" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F6"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F14"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>